<commit_message>
Add Points-by-Floor + LCP-to-Physical sheets to BMS I/O list
Points-by-Floor accounts for the full 4,467 physical points across the 67
panels (by floor + per-panel detail). LCP-to-Physical maps each of the 12
logical LCP groupings to the physical RS/RCP/CP panel(s) carrying its
equipment (equipment-served bridge) with coverage %, plus engineering-
judgement hints for the plant/DHC/lighting panels that carry no equip tag.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/exports/Red5-DHCP_BMS_IO_List.xlsx
+++ b/exports/Red5-DHCP_BMS_IO_List.xlsx
@@ -13,7 +13,9 @@
     <sheet name="IO_List" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="IO_Summary" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Reconciliation" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Legend" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Points-by-Floor" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="LCP-to-Physical" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Legend" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Panels'!$A$1:$F$13</definedName>
@@ -27,7 +29,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +61,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="13">
@@ -150,7 +156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -195,6 +201,10 @@
     <xf numFmtId="0" fontId="6" fillId="12" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -708,7 +718,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Panels · Controllers · IO_List (+ Phys. panel/floor cross-ref) · IO_Summary · Reconciliation · Legend</t>
+          <t>Panels · Controllers · IO_List (+ Phys. panel/floor cross-ref) · IO_Summary · Reconciliation · Points-by-Floor · LCP-to-Physical · Legend</t>
         </is>
       </c>
     </row>
@@ -86847,6 +86857,2322 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F86"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Physical panels accounting for the full 4,467 points (판넬별 포인트 정리 physical schedule)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The 4,467 installed I/O points live in 67 physical panels (RS/RCP/CP cabinets), grouped here by floor. The 1,160 functional points in this workbook are a drawing-derived subset bucketed into 12 logical LCP panels — see the LCP-to-Physical sheet for how they relate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Floor / area</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Panels</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Used points</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Capacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Penthouse (PH)</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>710</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>Floor 31</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="16" t="n">
+        <v>138</v>
+      </c>
+      <c r="D6" s="16" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Floor 21</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>152</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Floor 10</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>151</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Floor 4</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>492</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Floor 3</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>468</v>
+      </c>
+      <c r="D10" s="16" t="n">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Floor 2</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>458</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Floor 1</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="16" t="n">
+        <v>224</v>
+      </c>
+      <c r="D12" s="16" t="n">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Basement B1</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="C13" s="16" t="n">
+        <v>539</v>
+      </c>
+      <c r="D13" s="16" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Basement B2</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="C14" s="16" t="n">
+        <v>860</v>
+      </c>
+      <c r="D14" s="16" t="n">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Basement B3</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>275</v>
+      </c>
+      <c r="D15" s="16" t="n">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="n">
+        <v>67</v>
+      </c>
+      <c r="C16" s="17" t="n">
+        <v>4467</v>
+      </c>
+      <c r="D16" s="17" t="n">
+        <v>5240</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="20" t="inlineStr">
+        <is>
+          <t>Per-panel detail (67 physical panels)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="21" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="inlineStr">
+        <is>
+          <t>Panel</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="inlineStr">
+        <is>
+          <t>Floor</t>
+        </is>
+      </c>
+      <c r="D19" s="21" t="inlineStr">
+        <is>
+          <t>Equipment served</t>
+        </is>
+      </c>
+      <c r="E19" s="21" t="inlineStr">
+        <is>
+          <t>Used</t>
+        </is>
+      </c>
+      <c r="F19" s="21" t="inlineStr">
+        <is>
+          <t>Cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>RS-PH2-1</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>PH2</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr"/>
+      <c r="E20" s="6" t="n">
+        <v>66</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>RS-PH1-3</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>PH1</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr"/>
+      <c r="E21" s="6" t="n">
+        <v>165</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>CP-PH1-3</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>PH1</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr"/>
+      <c r="E22" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>CP-R-1</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>PH1</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr"/>
+      <c r="E23" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>RCP-PH1-3</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>PH1</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr"/>
+      <c r="E24" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>RCP-PH1-2</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>PH1</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>AC-24, EVU-11, EVU-13</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>116</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>RCP-PH1-1</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>PH1</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>AC-22, AC-23. EVU-15</t>
+        </is>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>CP-PH-1</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>PH1</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr"/>
+      <c r="E27" s="6" t="n">
+        <v>65</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="B28" s="6" t="inlineStr">
+        <is>
+          <t>RS-PH1-1</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>PH1</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr"/>
+      <c r="E28" s="6" t="n">
+        <v>88</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>RS-31-1</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>31F</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr"/>
+      <c r="E29" s="6" t="n">
+        <v>138</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>RS-21-1</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>21F</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr"/>
+      <c r="E30" s="6" t="n">
+        <v>152</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>RS-10-1</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>10F</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr"/>
+      <c r="E31" s="6" t="n">
+        <v>151</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>RCP-4-1</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>4F</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>EVU-8</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>RCP-4-2</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>4F</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>AC-17, AC-21, EVU-9</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>96</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B34" s="6" t="inlineStr">
+        <is>
+          <t>RCP-4-3</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>4F</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>AC-20, EVU-10</t>
+        </is>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="B35" s="6" t="inlineStr">
+        <is>
+          <t>RCP-4-4</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>4F</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>AC-18, AC-19</t>
+        </is>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n">
+        <v>17</v>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>CP-4-4</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>4F</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr"/>
+      <c r="E36" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>RS-4-1</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>4F</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr"/>
+      <c r="E37" s="6" t="n">
+        <v>102</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>RS-4-2</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>4F</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr"/>
+      <c r="E38" s="6" t="n">
+        <v>136</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>RCP-3-1</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>3F</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>AC-14</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n">
+        <v>21</v>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>RCP-3-2</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>3F</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>AC-15, AC-16, EVU-7</t>
+        </is>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="F40" s="6" t="n">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n">
+        <v>22</v>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>RS-3-1</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>3F</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="inlineStr"/>
+      <c r="E41" s="6" t="n">
+        <v>112</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>RS-3-2A</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>3F</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="inlineStr"/>
+      <c r="E42" s="6" t="n">
+        <v>172</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>RS-3-2B</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>3F</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="inlineStr"/>
+      <c r="E43" s="6" t="n">
+        <v>70</v>
+      </c>
+      <c r="F43" s="6" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>RCP-2-2</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>2F</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>AC-11, AC-12, AC-13, EVU-4, EVU-5</t>
+        </is>
+      </c>
+      <c r="E44" s="6" t="n">
+        <v>149</v>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="B45" s="6" t="inlineStr">
+        <is>
+          <t>RCP-2-3</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>2F</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="inlineStr"/>
+      <c r="E45" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="F45" s="6" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>RS-2-1</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>2F</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr"/>
+      <c r="E46" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="F46" s="6" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="B47" s="6" t="inlineStr">
+        <is>
+          <t>RS-2-2</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>2F</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr"/>
+      <c r="E47" s="6" t="n">
+        <v>102</v>
+      </c>
+      <c r="F47" s="6" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="B48" s="6" t="inlineStr">
+        <is>
+          <t>RS-2-3</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>2F</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr"/>
+      <c r="E48" s="6" t="n">
+        <v>96</v>
+      </c>
+      <c r="F48" s="6" t="n">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B49" s="6" t="inlineStr">
+        <is>
+          <t>EVU-6</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>2F</t>
+        </is>
+      </c>
+      <c r="D49" s="6" t="inlineStr"/>
+      <c r="E49" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F49" s="6" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>RCP-1-1</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>1F</t>
+        </is>
+      </c>
+      <c r="D50" s="6" t="inlineStr">
+        <is>
+          <t>EVU-1</t>
+        </is>
+      </c>
+      <c r="E50" s="6" t="n">
+        <v>23</v>
+      </c>
+      <c r="F50" s="6" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="B51" s="6" t="inlineStr">
+        <is>
+          <t>RCP-1-2</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>1F</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>AC-7, EVU-2</t>
+        </is>
+      </c>
+      <c r="E51" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="F51" s="6" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>RCP-1-3</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>1F</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>EVU-3</t>
+        </is>
+      </c>
+      <c r="E52" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="F52" s="6" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="B53" s="6" t="inlineStr">
+        <is>
+          <t>RS-1-1</t>
+        </is>
+      </c>
+      <c r="C53" s="6" t="inlineStr">
+        <is>
+          <t>1F</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr"/>
+      <c r="E53" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="F53" s="6" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="B54" s="6" t="inlineStr">
+        <is>
+          <t>RS-1-2</t>
+        </is>
+      </c>
+      <c r="C54" s="6" t="inlineStr">
+        <is>
+          <t>1F</t>
+        </is>
+      </c>
+      <c r="D54" s="6" t="inlineStr"/>
+      <c r="E54" s="6" t="n">
+        <v>73</v>
+      </c>
+      <c r="F54" s="6" t="n">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>RCP-B1-1</t>
+        </is>
+      </c>
+      <c r="C55" s="6" t="inlineStr">
+        <is>
+          <t>B1F</t>
+        </is>
+      </c>
+      <c r="D55" s="6" t="inlineStr">
+        <is>
+          <t>AC-5</t>
+        </is>
+      </c>
+      <c r="E55" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="F55" s="6" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>RCP-B1-2</t>
+        </is>
+      </c>
+      <c r="C56" s="6" t="inlineStr">
+        <is>
+          <t>B1F</t>
+        </is>
+      </c>
+      <c r="D56" s="6" t="inlineStr">
+        <is>
+          <t>AC-2, AC-2 (CO2), AC-6</t>
+        </is>
+      </c>
+      <c r="E56" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="F56" s="6" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>RCP-B1-3</t>
+        </is>
+      </c>
+      <c r="C57" s="6" t="inlineStr">
+        <is>
+          <t>B1F</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>AC-4</t>
+        </is>
+      </c>
+      <c r="E57" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="F57" s="6" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>RCP-B1-4</t>
+        </is>
+      </c>
+      <c r="C58" s="6" t="inlineStr">
+        <is>
+          <t>B1F</t>
+        </is>
+      </c>
+      <c r="D58" s="6" t="inlineStr">
+        <is>
+          <t>AC-2</t>
+        </is>
+      </c>
+      <c r="E58" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="F58" s="6" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>RCP-B1-5</t>
+        </is>
+      </c>
+      <c r="C59" s="6" t="inlineStr">
+        <is>
+          <t>B1F</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>PCU-11, PCU-13</t>
+        </is>
+      </c>
+      <c r="E59" s="6" t="n">
+        <v>26</v>
+      </c>
+      <c r="F59" s="6" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>CP-B1-2</t>
+        </is>
+      </c>
+      <c r="C60" s="6" t="inlineStr">
+        <is>
+          <t>B1F</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>PCU-8, PCU-9, PCU-10</t>
+        </is>
+      </c>
+      <c r="E60" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="F60" s="6" t="n">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="B61" s="6" t="inlineStr">
+        <is>
+          <t>CP-B1-3</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>B1F</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr"/>
+      <c r="E61" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F61" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="n">
+        <v>43</v>
+      </c>
+      <c r="B62" s="6" t="inlineStr">
+        <is>
+          <t>CP-B1-4</t>
+        </is>
+      </c>
+      <c r="C62" s="6" t="inlineStr">
+        <is>
+          <t>B1F</t>
+        </is>
+      </c>
+      <c r="D62" s="6" t="inlineStr">
+        <is>
+          <t>PCU-5, PCU-6, PCU-7-1, PCU-7-2</t>
+        </is>
+      </c>
+      <c r="E62" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="F62" s="6" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="n">
+        <v>44</v>
+      </c>
+      <c r="B63" s="6" t="inlineStr">
+        <is>
+          <t>RS-B1-1</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>B1F</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr"/>
+      <c r="E63" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="F63" s="6" t="n">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="n">
+        <v>45</v>
+      </c>
+      <c r="B64" s="6" t="inlineStr">
+        <is>
+          <t>RS-B1-2</t>
+        </is>
+      </c>
+      <c r="C64" s="6" t="inlineStr">
+        <is>
+          <t>B1F</t>
+        </is>
+      </c>
+      <c r="D64" s="6" t="inlineStr"/>
+      <c r="E64" s="6" t="n">
+        <v>114</v>
+      </c>
+      <c r="F64" s="6" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="n">
+        <v>46</v>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>RS-B1-3</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>B1F</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr"/>
+      <c r="E65" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="F65" s="6" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="n">
+        <v>47</v>
+      </c>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>시스템 제어반</t>
+        </is>
+      </c>
+      <c r="C66" s="6" t="inlineStr">
+        <is>
+          <t>B2F</t>
+        </is>
+      </c>
+      <c r="D66" s="6" t="inlineStr"/>
+      <c r="E66" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="F66" s="6" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>RCP-B2-1</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>B2F</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>AC-3</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="n">
+        <v>29</v>
+      </c>
+      <c r="F67" s="6" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="n">
+        <v>49</v>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>RCP-B2-2</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>B2F</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>SF-10, SF-11, EF-10, EF-11</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="F68" s="6" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>RCP-B2-3</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>B2F</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>SF-12, EF-12</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="F69" s="6" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="n">
+        <v>51</v>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>RCP-B2-4</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>B2F</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr"/>
+      <c r="E70" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F70" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="n">
+        <v>52</v>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>CP-B2-3</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>B2F</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>AC-26</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="F71" s="6" t="n">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="n">
+        <v>53</v>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>CP-B2-4</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>B2F</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr"/>
+      <c r="E72" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="F72" s="6" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>RS-B2-1</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>B2F</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr"/>
+      <c r="E73" s="6" t="n">
+        <v>76</v>
+      </c>
+      <c r="F73" s="6" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="n">
+        <v>55</v>
+      </c>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>RS-B2-2</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>B2F</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr"/>
+      <c r="E74" s="6" t="n">
+        <v>78</v>
+      </c>
+      <c r="F74" s="6" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>RS-B2-3</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>B2F</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr"/>
+      <c r="E75" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="F75" s="6" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="n">
+        <v>57</v>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>RS-B2-4B</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>B2F</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr"/>
+      <c r="E76" s="6" t="n">
+        <v>124</v>
+      </c>
+      <c r="F76" s="6" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>RS-B2-4A</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>B2F</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr"/>
+      <c r="E77" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="F77" s="6" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>RS-B2-5</t>
+        </is>
+      </c>
+      <c r="C78" s="6" t="inlineStr">
+        <is>
+          <t>B2F</t>
+        </is>
+      </c>
+      <c r="D78" s="6" t="inlineStr"/>
+      <c r="E78" s="6" t="n">
+        <v>97</v>
+      </c>
+      <c r="F78" s="6" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="n">
+        <v>60</v>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>RS-B2-6</t>
+        </is>
+      </c>
+      <c r="C79" s="6" t="inlineStr">
+        <is>
+          <t>B2F</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr"/>
+      <c r="E79" s="6" t="n">
+        <v>83</v>
+      </c>
+      <c r="F79" s="6" t="n">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="n">
+        <v>61</v>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>RS-B2-7</t>
+        </is>
+      </c>
+      <c r="C80" s="6" t="inlineStr">
+        <is>
+          <t>B2F</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr"/>
+      <c r="E80" s="6" t="n">
+        <v>129</v>
+      </c>
+      <c r="F80" s="6" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="n">
+        <v>62</v>
+      </c>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>P-1</t>
+        </is>
+      </c>
+      <c r="C81" s="6" t="inlineStr">
+        <is>
+          <t>B2F or B3F (추정)</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr"/>
+      <c r="E81" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F81" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>RCP-B3-1</t>
+        </is>
+      </c>
+      <c r="C82" s="6" t="inlineStr">
+        <is>
+          <t>B3F</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>AC-1</t>
+        </is>
+      </c>
+      <c r="E82" s="6" t="n">
+        <v>28</v>
+      </c>
+      <c r="F82" s="6" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="n">
+        <v>64</v>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>RCP-B3-2</t>
+        </is>
+      </c>
+      <c r="C83" s="6" t="inlineStr">
+        <is>
+          <t>B3F</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>SF-3, EF-2</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="F83" s="6" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="n">
+        <v>65</v>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>RCP-B3-3</t>
+        </is>
+      </c>
+      <c r="C84" s="6" t="inlineStr">
+        <is>
+          <t>B3F</t>
+        </is>
+      </c>
+      <c r="D84" s="6" t="inlineStr">
+        <is>
+          <t>SF-4, SF-5, EF-3, EF-4</t>
+        </is>
+      </c>
+      <c r="E84" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="F84" s="6" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="n">
+        <v>66</v>
+      </c>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>CP-B3-2</t>
+        </is>
+      </c>
+      <c r="C85" s="6" t="inlineStr">
+        <is>
+          <t>B3F</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr"/>
+      <c r="E85" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="F85" s="6" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="n">
+        <v>67</v>
+      </c>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>RS-B3-1</t>
+        </is>
+      </c>
+      <c r="C86" s="6" t="inlineStr">
+        <is>
+          <t>B3F</t>
+        </is>
+      </c>
+      <c r="D86" s="6" t="inlineStr"/>
+      <c r="E86" s="6" t="n">
+        <v>167</v>
+      </c>
+      <c r="F86" s="6" t="n">
+        <v>172</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="46" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Logical (LCP) panels → physical panels</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Each functional LCP grouping mapped to the physical RS/RCP/CP panel(s) that carry its equipment, via the equipment-served bridge. Plant / DHC / metering / lighting devices are not equipment-tagged in the physical schedule, so those rows show the drawing location + an engineering-judgement hint instead of a hard match.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="21" t="inlineStr">
+        <is>
+          <t>LCP panel</t>
+        </is>
+      </c>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Drawing location</t>
+        </is>
+      </c>
+      <c r="C4" s="21" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="D4" s="21" t="inlineStr">
+        <is>
+          <t>Matched physical panels (floor)</t>
+        </is>
+      </c>
+      <c r="E4" s="21" t="inlineStr">
+        <is>
+          <t>Linked pts</t>
+        </is>
+      </c>
+      <c r="F4" s="21" t="inlineStr">
+        <is>
+          <t>Coverage</t>
+        </is>
+      </c>
+      <c r="G4" s="21" t="inlineStr">
+        <is>
+          <t>Note (engineering judgement)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>BMS-CENTRAL</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>B2F Central Monitoring Rm</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G5" s="6">
+        <f> 시스템 제어반 (B2F) — the physical central/system panel</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>LCP-DHC</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>B2F Machine Room</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>56</v>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>DHC intake devices in B2F machine-room CP-* panels (not equip-tagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>LCP-CT</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Rooftop / PH</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>83</v>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Tower/condenser devices on rooftop / PH plant panels (not equip-tagged)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>LCP-HSL</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>B2F Machine Room</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>222</v>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>CP-B2-3 (B2F), RCP-B1-1 (B1F), RCP-B1-2 (B1F), RCP-B1-3 (B1F), RCP-B2-1 (B2F), RCP-B3-1 (B3F)</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>75</v>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>33%</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>Low-rise CHW/HW pumps + HX in basement machine-room CP-* panels</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>LCP-HSH</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>PH Machine Room</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>182</v>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>RCP-PH1-1 (PH1), RCP-PH1-2 (PH1)</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>High-rise + 36/37F pumps/HX incl. R-1 → CP-R-1 (PH1) + basement CP-*</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>LCP-3637</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>37F PH Machine Room</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>171</v>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>RCP-PH1-1 (PH1), RCP-PH1-2 (PH1)</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>LCP-1F</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>1F EPS/AHU Room</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="n">
+        <v>54</v>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>RCP-1-1 (1F), RCP-1-2 (1F), RCP-1-3 (1F)</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>48</v>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>88%</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>LCP-2F</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>2F AHU Room</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="n">
+        <v>117</v>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>RCP-2-2 (2F), RCP-B3-2 (B3F)</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>63</v>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>53%</t>
+        </is>
+      </c>
+      <c r="G12" s="6" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>LCP-3F</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
+        <is>
+          <t>3F AHU Room</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="n">
+        <v>68</v>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>RCP-3-1 (3F), RCP-3-2 (3F)</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>73%</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="inlineStr">
+        <is>
+          <t>LCP-4F</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
+        <is>
+          <t>4F AHU Room</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>133</v>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>RCP-4-1 (4F), RCP-4-2 (4F), RCP-4-3 (4F), RCP-4-4 (4F)</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>101</v>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>75%</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>LCP-PKG</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>B3F–B1F EPS</t>
+        </is>
+      </c>
+      <c r="C15" s="6" t="n">
+        <v>58</v>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>CP-B1-2 (B1F), CP-B1-4 (B1F), RCP-B1-5 (B1F)</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>18</v>
+      </c>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>31%</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Packaged units → CP-B1-2 / CP-B1-4 / RCP-B1-5 (PCU tags)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>LCP-LTG</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Distributed EPS</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="6" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>Common-area/facade lighting distributed across RS-* room panels</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -86867,7 +89193,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>AI</t>
         </is>
@@ -86879,7 +89205,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="20" t="inlineStr">
+      <c r="A3" s="22" t="inlineStr">
         <is>
           <t>AO</t>
         </is>
@@ -86891,7 +89217,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="22" t="inlineStr">
         <is>
           <t>BI</t>
         </is>
@@ -86903,7 +89229,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>BO</t>
         </is>
@@ -86915,7 +89241,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>SP/Sched</t>
         </is>
@@ -86927,7 +89253,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="22" t="inlineStr">
         <is>
           <t>CHW / CW</t>
         </is>
@@ -86939,7 +89265,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="22" t="inlineStr">
         <is>
           <t>SAT / RAT</t>
         </is>
@@ -86951,7 +89277,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>CCV / HCV</t>
         </is>
@@ -86963,7 +89289,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>INV</t>
         </is>
@@ -86975,7 +89301,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>Zero-energy band</t>
         </is>
@@ -86987,7 +89313,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>DHC</t>
         </is>
@@ -86999,7 +89325,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>HEX / EX</t>
         </is>
@@ -87011,7 +89337,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>EX-1</t>
         </is>
@@ -87023,7 +89349,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>CS / CR</t>
         </is>
@@ -87035,7 +89361,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>SS / HR</t>
         </is>
@@ -87047,7 +89373,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="inlineStr">
+      <c r="A17" s="22" t="inlineStr">
         <is>
           <t>R-1</t>
         </is>
@@ -87059,7 +89385,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>CDP</t>
         </is>
@@ -87071,7 +89397,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="20" t="inlineStr">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>CP / HP</t>
         </is>
@@ -87083,7 +89409,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="inlineStr">
+      <c r="A20" s="22" t="inlineStr">
         <is>
           <t>CT</t>
         </is>
@@ -87095,7 +89421,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>HWT-1</t>
         </is>
@@ -87107,7 +89433,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="20" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>PCU/PAC/PMAC</t>
         </is>
@@ -87119,7 +89445,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>OAU (EVU)</t>
         </is>
@@ -87131,7 +89457,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="20" t="inlineStr">
+      <c r="A24" s="22" t="inlineStr">
         <is>
           <t>順序 / 群起動</t>
         </is>

</xml_diff>

<commit_message>
Document best-effort bridge caveat on LCP-to-Physical sheet
Adds a "How to read this" note explaining the equipment-tag mapping is
best-effort (high for air-side LCPs, 0% for untagged plant/DHC/lighting)
and flags possible cross-floor tag coincidences to verify against drawings.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/exports/Red5-DHCP_BMS_IO_List.xlsx
+++ b/exports/Red5-DHCP_BMS_IO_List.xlsx
@@ -88724,7 +88724,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -89159,6 +89159,18 @@
       <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Common-area/facade lighting distributed across RS-* room panels</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="96" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>How to read this</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>The 'Matched physical panels' column is a BEST-EFFORT bridge: a functional device (e.g. AC-17) is linked to a physical panel only when that panel's 'equipment served' column names the same tag. So coverage is high for the air-side floor LCPs (AHUs/OAUs) and partial elsewhere. Rows at 0% coverage (BMS-CENTRAL, LCP-DHC, LCP-CT, LCP-LTG) hold plant / DHC / metering / lighting points that are NOT equipment-tagged in the physical schedule — use the drawing location + judgement note for those. Caveat: matching is by tag string only, so a repeated fan/unit number can produce a cross-floor coincidence (e.g. a 2F SF tag also appearing on a basement fan panel) — verify against the drawings before relying on a single-panel assignment.</t>
         </is>
       </c>
     </row>

</xml_diff>